<commit_message>
fix: bugs catalogo v3.1.0 (FLG_INACTIVO, safe-float, ean, un_bx stats, backup race, duplicados) + BAT --auto con retry y X-API-Key + tests v3 + README
</commit_message>
<xml_diff>
--- a/data/SKU_BX.xlsx
+++ b/data/SKU_BX.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccusi\Documents\Proyect_Coder\G360-ecosystem\projects\g360-master-data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8847D019-68DD-4635-826D-49094D35CE90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700C223B-FBFD-40F6-B2F5-102433851780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6300" yWindow="1710" windowWidth="20865" windowHeight="11055" xr2:uid="{B19518BF-BEE8-4C61-8490-6B34AC0E6445}"/>
+    <workbookView xWindow="9840" yWindow="240" windowWidth="11940" windowHeight="11565" xr2:uid="{B19518BF-BEE8-4C61-8490-6B34AC0E6445}"/>
   </bookViews>
   <sheets>
     <sheet name="SKU_BX" sheetId="1" r:id="rId1"/>
@@ -11761,7 +11761,7 @@
         <v>1006</v>
       </c>
       <c r="C588">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="D588" t="s">
         <v>968</v>
@@ -11775,7 +11775,7 @@
         <v>1007</v>
       </c>
       <c r="C589">
-        <v>576</v>
+        <v>28</v>
       </c>
       <c r="D589" t="s">
         <v>968</v>
@@ -11789,7 +11789,7 @@
         <v>1008</v>
       </c>
       <c r="C590">
-        <v>576</v>
+        <v>28</v>
       </c>
       <c r="D590" t="s">
         <v>968</v>
@@ -11803,7 +11803,7 @@
         <v>1009</v>
       </c>
       <c r="C591">
-        <v>576</v>
+        <v>28</v>
       </c>
       <c r="D591" t="s">
         <v>968</v>
@@ -11817,7 +11817,7 @@
         <v>1010</v>
       </c>
       <c r="C592">
-        <v>576</v>
+        <v>28</v>
       </c>
       <c r="D592" t="s">
         <v>968</v>
@@ -11831,7 +11831,7 @@
         <v>1011</v>
       </c>
       <c r="C593">
-        <v>576</v>
+        <v>28</v>
       </c>
       <c r="D593" t="s">
         <v>968</v>
@@ -12265,7 +12265,7 @@
         <v>1016</v>
       </c>
       <c r="C624">
-        <v>576</v>
+        <v>144</v>
       </c>
       <c r="D624" t="s">
         <v>968</v>
@@ -12279,7 +12279,7 @@
         <v>1017</v>
       </c>
       <c r="C625">
-        <v>576</v>
+        <v>144</v>
       </c>
       <c r="D625" t="s">
         <v>968</v>
@@ -12293,7 +12293,7 @@
         <v>1018</v>
       </c>
       <c r="C626">
-        <v>576</v>
+        <v>144</v>
       </c>
       <c r="D626" t="s">
         <v>968</v>

</xml_diff>